<commit_message>
Add edge-case sample data and handle blanks and duplicates in analysis
</commit_message>
<xml_diff>
--- a/data/offers.xlsx
+++ b/data/offers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,6 +514,104 @@
         <v>800</v>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>Loyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OF-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Early-access discount</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>400</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Loyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OF-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Free premium upgrade</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Loyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OF-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Surprise gift</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Loyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OF-4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Early-access discount</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>400</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>

</xml_diff>

<commit_message>
Extend offers sample to 15 rows and add budgets for Premium
</commit_message>
<xml_diff>
--- a/data/offers.xlsx
+++ b/data/offers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,6 +614,206 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>Loyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>OF-7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Premium early renewal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>500</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OF-8</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Priority support credit</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>700</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OF-9</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Anniversary discount</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>900</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OF-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Concierge review</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OF-11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bundle upgrade</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OF-12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Loyalty reward plus</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OF-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Extended warranty</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>450</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OF-14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Exclusive event access</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Premium</t>
         </is>
       </c>
     </row>
@@ -628,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -673,6 +873,16 @@
         <v>2000</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>